<commit_message>
fix: limpiar response del detalle de producto — quitar campos innecesarios
</commit_message>
<xml_diff>
--- a/productos.xlsx
+++ b/productos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/charlyboyapple/bellezagdl-backend/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8296370E-9286-9A46-AFB5-8DC71F97A88B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B362C0F8-88B1-3C4A-8285-A6336D6287E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31220" yWindow="7140" windowWidth="27140" windowHeight="12560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="36820" yWindow="10640" windowWidth="31240" windowHeight="13460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="43">
   <si>
     <t>Alby</t>
   </si>
@@ -147,6 +147,21 @@
   </si>
   <si>
     <t>Algodón Plisado 100gr Alby</t>
+  </si>
+  <si>
+    <t>01 Rojo</t>
+  </si>
+  <si>
+    <t>02 Blanco</t>
+  </si>
+  <si>
+    <t>A50G_01</t>
+  </si>
+  <si>
+    <t>A50G_02</t>
+  </si>
+  <si>
+    <t>no</t>
   </si>
 </sst>
 </file>
@@ -508,18 +523,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="37.33203125" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.5" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="34.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.83203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="29" style="2" customWidth="1"/>
+    <col min="4" max="4" width="7.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.6640625" style="2" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8.6640625" style="2" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="16.1640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="37.33203125" style="2"/>
+    <col min="9" max="9" width="6.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.83203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="37.33203125" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
@@ -644,7 +661,7 @@
         <v>10</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>34</v>
@@ -658,19 +675,19 @@
         <v>1</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G5" s="2">
-        <v>32</v>
+        <v>13.2</v>
       </c>
       <c r="H5" s="2">
         <v>10</v>
@@ -679,7 +696,7 @@
         <v>24</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="15" x14ac:dyDescent="0.2">
@@ -690,19 +707,19 @@
         <v>1</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>10</v>
+        <v>41</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G6" s="2">
-        <v>17.7</v>
+        <v>13.2</v>
       </c>
       <c r="H6" s="2">
         <v>10</v>
@@ -722,19 +739,19 @@
         <v>1</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>22</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F7" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G7" s="2">
         <v>32</v>
-      </c>
-      <c r="G7" s="2">
-        <v>25</v>
       </c>
       <c r="H7" s="2">
         <v>10</v>
@@ -743,7 +760,7 @@
         <v>24</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="15" x14ac:dyDescent="0.2">
@@ -754,19 +771,19 @@
         <v>1</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>22</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="G8" s="2">
-        <v>21.3</v>
+        <v>17.7</v>
       </c>
       <c r="H8" s="2">
         <v>10</v>
@@ -775,6 +792,70 @@
         <v>24</v>
       </c>
       <c r="J8" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="15" x14ac:dyDescent="0.2">
+      <c r="A9" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G9" s="2">
+        <v>25</v>
+      </c>
+      <c r="H9" s="2">
+        <v>10</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="15" x14ac:dyDescent="0.2">
+      <c r="A10" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G10" s="2">
+        <v>21.3</v>
+      </c>
+      <c r="H10" s="2">
+        <v>10</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J10" s="2" t="s">
         <v>34</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: rol oferta — catalogo filtrado con precios especiales para clientes de oferta
</commit_message>
<xml_diff>
--- a/productos.xlsx
+++ b/productos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/charlyboyapple/bellezagdl-backend/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFAA95BE-2A93-9C4C-9764-7BAA535FAA66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD91EBE6-629D-874C-8346-4DDDC1498EC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15700" yWindow="4800" windowWidth="31240" windowHeight="13460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="29360" yWindow="5500" windowWidth="31240" windowHeight="13460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1034" uniqueCount="258">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1041" uniqueCount="260">
   <si>
     <t>Alby</t>
   </si>
@@ -807,6 +807,12 @@
   </si>
   <si>
     <t>no</t>
+  </si>
+  <si>
+    <t>oferta</t>
+  </si>
+  <si>
+    <t>precio_oferta</t>
   </si>
 </sst>
 </file>
@@ -1179,7 +1185,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J129"/>
+  <dimension ref="A1:L129"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="37.33203125" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.33203125" style="1" customWidth="1"/>
@@ -1192,10 +1198,12 @@
     <col min="8" max="8" width="16.1640625" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="6.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="12.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="37.33203125" style="1"/>
+    <col min="11" max="11" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="37.33203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>6</v>
       </c>
@@ -1226,8 +1234,14 @@
       <c r="J1" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K1" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1258,8 +1272,14 @@
       <c r="J2" s="1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="L2" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -1290,8 +1310,14 @@
       <c r="J3" s="1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="L3" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>19</v>
       </c>
@@ -1322,8 +1348,14 @@
       <c r="J4" s="1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="L4" s="1">
+        <v>40.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>23</v>
       </c>
@@ -1355,7 +1387,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>23</v>
       </c>
@@ -1387,7 +1419,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>19</v>
       </c>
@@ -1418,8 +1450,14 @@
       <c r="J7" s="1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="L7" s="1">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>19</v>
       </c>
@@ -1451,7 +1489,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>19</v>
       </c>
@@ -1483,7 +1521,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>19</v>
       </c>
@@ -1515,7 +1553,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>19</v>
       </c>
@@ -1547,7 +1585,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>19</v>
       </c>
@@ -1579,7 +1617,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>19</v>
       </c>
@@ -1611,7 +1649,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>19</v>
       </c>
@@ -1643,7 +1681,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>23</v>
       </c>
@@ -1674,8 +1712,14 @@
       <c r="J15" s="1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K15" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="L15" s="1">
+        <v>99.4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>23</v>
       </c>

</xml_diff>